<commit_message>
Update total intervention contact event duration in BCIO_Schedule.xlsx
</commit_message>
<xml_diff>
--- a/Schedule/BCIO_Schedule.xlsx
+++ b/Schedule/BCIO_Schedule.xlsx
@@ -531,27 +531,27 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
+          <t>Curator</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
           <t>Curation status</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Definition_ID</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>To be reviewed by</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>Definition_ID</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Reviewer query</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>Curator</t>
         </is>
       </c>
     </row>
@@ -595,12 +595,12 @@
       <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="n"/>
       <c r="S2" s="2" t="n"/>
-      <c r="T2" s="2" t="inlineStr">
+      <c r="T2" s="2" t="n"/>
+      <c r="U2" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U2" s="2" t="n"/>
       <c r="V2" s="2" t="n"/>
       <c r="W2" s="2" t="n"/>
       <c r="X2" s="2" t="n"/>
@@ -628,12 +628,12 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
+          <t>JH; PS</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>JH; PS</t>
         </is>
       </c>
     </row>
@@ -709,21 +709,21 @@
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
+          <t>CM; JH; PS</t>
+        </is>
+      </c>
+      <c r="U4" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U4" s="2" t="inlineStr">
+      <c r="V4" s="2" t="n"/>
+      <c r="W4" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="V4" s="2" t="n"/>
-      <c r="W4" s="2" t="n"/>
-      <c r="X4" s="2" t="inlineStr">
-        <is>
-          <t>CM; JH; PS</t>
-        </is>
-      </c>
+      <c r="X4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -761,12 +761,12 @@
       <c r="Q5" s="3" t="n"/>
       <c r="R5" s="3" t="n"/>
       <c r="S5" s="3" t="n"/>
-      <c r="T5" s="3" t="inlineStr">
+      <c r="T5" s="3" t="n"/>
+      <c r="U5" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U5" s="3" t="n"/>
       <c r="V5" s="3" t="n"/>
       <c r="W5" s="3" t="n"/>
       <c r="X5" s="3" t="n"/>
@@ -807,12 +807,12 @@
       <c r="Q6" s="2" t="n"/>
       <c r="R6" s="2" t="n"/>
       <c r="S6" s="2" t="n"/>
-      <c r="T6" s="2" t="inlineStr">
+      <c r="T6" s="2" t="n"/>
+      <c r="U6" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U6" s="2" t="n"/>
       <c r="V6" s="2" t="n"/>
       <c r="W6" s="2" t="n"/>
       <c r="X6" s="2" t="n"/>
@@ -868,17 +868,17 @@
       <c r="S7" s="2" t="n"/>
       <c r="T7" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U7" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U7" s="2" t="n"/>
       <c r="V7" s="2" t="n"/>
       <c r="W7" s="2" t="n"/>
-      <c r="X7" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -916,12 +916,12 @@
       <c r="Q8" s="3" t="n"/>
       <c r="R8" s="3" t="n"/>
       <c r="S8" s="3" t="n"/>
-      <c r="T8" s="3" t="inlineStr">
+      <c r="T8" s="3" t="n"/>
+      <c r="U8" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U8" s="3" t="n"/>
       <c r="V8" s="3" t="n"/>
       <c r="W8" s="3" t="n"/>
       <c r="X8" s="3" t="n"/>
@@ -972,17 +972,17 @@
       <c r="S9" s="2" t="n"/>
       <c r="T9" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U9" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U9" s="2" t="n"/>
       <c r="V9" s="2" t="n"/>
       <c r="W9" s="2" t="n"/>
-      <c r="X9" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1020,12 +1020,12 @@
       <c r="Q10" s="3" t="n"/>
       <c r="R10" s="3" t="n"/>
       <c r="S10" s="3" t="n"/>
-      <c r="T10" s="3" t="inlineStr">
+      <c r="T10" s="3" t="n"/>
+      <c r="U10" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U10" s="3" t="n"/>
       <c r="V10" s="3" t="n"/>
       <c r="W10" s="3" t="n"/>
       <c r="X10" s="3" t="n"/>
@@ -1076,17 +1076,17 @@
       <c r="S11" s="2" t="n"/>
       <c r="T11" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U11" s="2" t="n"/>
       <c r="V11" s="2" t="n"/>
       <c r="W11" s="2" t="n"/>
-      <c r="X11" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1147,17 +1147,17 @@
       <c r="S12" s="2" t="n"/>
       <c r="T12" s="2" t="inlineStr">
         <is>
+          <t>CM; JH; PS</t>
+        </is>
+      </c>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U12" s="2" t="n"/>
       <c r="V12" s="2" t="n"/>
       <c r="W12" s="2" t="n"/>
-      <c r="X12" s="2" t="inlineStr">
-        <is>
-          <t>CM; JH; PS</t>
-        </is>
-      </c>
+      <c r="X12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1195,12 +1195,12 @@
       <c r="Q13" s="3" t="n"/>
       <c r="R13" s="3" t="n"/>
       <c r="S13" s="3" t="n"/>
-      <c r="T13" s="3" t="inlineStr">
+      <c r="T13" s="3" t="n"/>
+      <c r="U13" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U13" s="3" t="n"/>
       <c r="V13" s="3" t="n"/>
       <c r="W13" s="3" t="n"/>
       <c r="X13" s="3" t="n"/>
@@ -1251,17 +1251,17 @@
       <c r="S14" s="2" t="n"/>
       <c r="T14" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U14" s="2" t="n"/>
       <c r="V14" s="2" t="n"/>
       <c r="W14" s="2" t="n"/>
-      <c r="X14" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1309,17 +1309,17 @@
       <c r="S15" s="2" t="n"/>
       <c r="T15" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U15" s="2" t="n"/>
       <c r="V15" s="2" t="n"/>
       <c r="W15" s="2" t="n"/>
-      <c r="X15" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1381,21 +1381,21 @@
       </c>
       <c r="T16" s="2" t="inlineStr">
         <is>
+          <t>CM; RW; JH; PS</t>
+        </is>
+      </c>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U16" s="2" t="inlineStr">
+      <c r="V16" s="2" t="n"/>
+      <c r="W16" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="V16" s="2" t="n"/>
-      <c r="W16" s="2" t="n"/>
-      <c r="X16" s="2" t="inlineStr">
-        <is>
-          <t>CM; RW; JH; PS</t>
-        </is>
-      </c>
+      <c r="X16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1433,12 +1433,12 @@
       <c r="Q17" s="3" t="n"/>
       <c r="R17" s="3" t="n"/>
       <c r="S17" s="3" t="n"/>
-      <c r="T17" s="3" t="inlineStr">
+      <c r="T17" s="3" t="n"/>
+      <c r="U17" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U17" s="3" t="n"/>
       <c r="V17" s="3" t="n"/>
       <c r="W17" s="3" t="n"/>
       <c r="X17" s="3" t="n"/>
@@ -1489,17 +1489,17 @@
       <c r="S18" s="2" t="n"/>
       <c r="T18" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U18" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U18" s="2" t="n"/>
       <c r="V18" s="2" t="n"/>
       <c r="W18" s="2" t="n"/>
-      <c r="X18" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1549,12 +1549,12 @@
       <c r="Q19" s="2" t="n"/>
       <c r="R19" s="2" t="n"/>
       <c r="S19" s="2" t="n"/>
-      <c r="T19" s="2" t="inlineStr">
+      <c r="T19" s="2" t="n"/>
+      <c r="U19" s="2" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U19" s="2" t="n"/>
       <c r="V19" s="2" t="n"/>
       <c r="W19" s="2" t="n"/>
       <c r="X19" s="2" t="n"/>
@@ -1605,17 +1605,17 @@
       <c r="S20" s="3" t="n"/>
       <c r="T20" s="3" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U20" s="3" t="inlineStr">
+        <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U20" s="3" t="n"/>
       <c r="V20" s="3" t="n"/>
       <c r="W20" s="3" t="n"/>
-      <c r="X20" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -1653,12 +1653,12 @@
       <c r="Q21" s="3" t="n"/>
       <c r="R21" s="3" t="n"/>
       <c r="S21" s="3" t="n"/>
-      <c r="T21" s="3" t="inlineStr">
+      <c r="T21" s="3" t="n"/>
+      <c r="U21" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U21" s="3" t="n"/>
       <c r="V21" s="3" t="n"/>
       <c r="W21" s="3" t="n"/>
       <c r="X21" s="3" t="n"/>
@@ -1728,21 +1728,21 @@
       <c r="S22" s="2" t="n"/>
       <c r="T22" s="2" t="inlineStr">
         <is>
+          <t>CM; EJH; PS</t>
+        </is>
+      </c>
+      <c r="U22" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U22" s="2" t="inlineStr">
+      <c r="V22" s="2" t="n"/>
+      <c r="W22" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="V22" s="2" t="n"/>
-      <c r="W22" s="2" t="n"/>
-      <c r="X22" s="2" t="inlineStr">
-        <is>
-          <t>CM; EJH; PS</t>
-        </is>
-      </c>
+      <c r="X22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -1780,12 +1780,12 @@
       <c r="Q23" s="3" t="n"/>
       <c r="R23" s="3" t="n"/>
       <c r="S23" s="3" t="n"/>
-      <c r="T23" s="3" t="inlineStr">
+      <c r="T23" s="3" t="n"/>
+      <c r="U23" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U23" s="3" t="n"/>
       <c r="V23" s="3" t="n"/>
       <c r="W23" s="3" t="n"/>
       <c r="X23" s="3" t="n"/>
@@ -1850,21 +1850,21 @@
       </c>
       <c r="T24" s="2" t="inlineStr">
         <is>
+          <t>CM; JH; PS</t>
+        </is>
+      </c>
+      <c r="U24" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U24" s="2" t="inlineStr">
+      <c r="V24" s="2" t="n"/>
+      <c r="W24" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="V24" s="2" t="n"/>
-      <c r="W24" s="2" t="n"/>
-      <c r="X24" s="2" t="inlineStr">
-        <is>
-          <t>CM; JH; PS</t>
-        </is>
-      </c>
+      <c r="X24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -1902,12 +1902,12 @@
       <c r="Q25" s="3" t="n"/>
       <c r="R25" s="3" t="n"/>
       <c r="S25" s="3" t="n"/>
-      <c r="T25" s="3" t="inlineStr">
+      <c r="T25" s="3" t="n"/>
+      <c r="U25" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U25" s="3" t="n"/>
       <c r="V25" s="3" t="n"/>
       <c r="W25" s="3" t="n"/>
       <c r="X25" s="3" t="n"/>
@@ -1958,17 +1958,17 @@
       <c r="S26" s="2" t="n"/>
       <c r="T26" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U26" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U26" s="2" t="n"/>
       <c r="V26" s="2" t="n"/>
       <c r="W26" s="2" t="n"/>
-      <c r="X26" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2030,17 +2030,17 @@
       <c r="S27" s="2" t="n"/>
       <c r="T27" s="2" t="inlineStr">
         <is>
+          <t>CM; JH; PS</t>
+        </is>
+      </c>
+      <c r="U27" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U27" s="2" t="n"/>
       <c r="V27" s="2" t="n"/>
       <c r="W27" s="2" t="n"/>
-      <c r="X27" s="2" t="inlineStr">
-        <is>
-          <t>CM; JH; PS</t>
-        </is>
-      </c>
+      <c r="X27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -2082,12 +2082,12 @@
       <c r="Q28" s="3" t="n"/>
       <c r="R28" s="3" t="n"/>
       <c r="S28" s="3" t="n"/>
-      <c r="T28" s="3" t="inlineStr">
+      <c r="T28" s="3" t="n"/>
+      <c r="U28" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U28" s="3" t="n"/>
       <c r="V28" s="3" t="n"/>
       <c r="W28" s="3" t="n"/>
       <c r="X28" s="3" t="n"/>
@@ -2138,17 +2138,17 @@
       <c r="S29" s="2" t="n"/>
       <c r="T29" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U29" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U29" s="2" t="n"/>
       <c r="V29" s="2" t="n"/>
       <c r="W29" s="2" t="n"/>
-      <c r="X29" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2205,23 +2205,23 @@
       <c r="S30" s="2" t="n"/>
       <c r="T30" s="2" t="inlineStr">
         <is>
+          <t>CM; JH; PS</t>
+        </is>
+      </c>
+      <c r="U30" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
-        </is>
-      </c>
-      <c r="U30" s="2" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="V30" s="2" t="n"/>
       <c r="W30" s="2" t="inlineStr">
         <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="X30" s="2" t="inlineStr">
+        <is>
           <t>should we also add separate entities for fixed and variable schedule, to describe cases when schedules vary across participants? We previously had these entities within the ontology but they were removed as they didn't come up explicitly in papers and our old definition of variable schedule overlapped with the definition for irregular schedule (CM)</t>
-        </is>
-      </c>
-      <c r="X30" s="2" t="inlineStr">
-        <is>
-          <t>CM; JH; PS</t>
         </is>
       </c>
     </row>
@@ -2274,12 +2274,12 @@
       <c r="Q31" s="3" t="n"/>
       <c r="R31" s="3" t="n"/>
       <c r="S31" s="3" t="n"/>
-      <c r="T31" s="3" t="inlineStr">
+      <c r="T31" s="3" t="n"/>
+      <c r="U31" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U31" s="3" t="n"/>
       <c r="V31" s="3" t="n"/>
       <c r="W31" s="3" t="n"/>
       <c r="X31" s="3" t="n"/>
@@ -2330,17 +2330,17 @@
       <c r="S32" s="2" t="n"/>
       <c r="T32" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U32" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U32" s="2" t="n"/>
       <c r="V32" s="2" t="n"/>
       <c r="W32" s="2" t="n"/>
-      <c r="X32" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2388,17 +2388,17 @@
       <c r="S33" s="2" t="n"/>
       <c r="T33" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U33" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U33" s="2" t="n"/>
       <c r="V33" s="2" t="n"/>
       <c r="W33" s="2" t="n"/>
-      <c r="X33" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2446,17 +2446,17 @@
       <c r="S34" s="2" t="n"/>
       <c r="T34" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U34" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U34" s="2" t="n"/>
       <c r="V34" s="2" t="n"/>
       <c r="W34" s="2" t="n"/>
-      <c r="X34" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2504,17 +2504,17 @@
       <c r="S35" s="2" t="n"/>
       <c r="T35" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U35" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U35" s="2" t="n"/>
       <c r="V35" s="2" t="n"/>
       <c r="W35" s="2" t="n"/>
-      <c r="X35" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2562,17 +2562,17 @@
       <c r="S36" s="2" t="n"/>
       <c r="T36" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U36" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U36" s="2" t="n"/>
       <c r="V36" s="2" t="n"/>
       <c r="W36" s="2" t="n"/>
-      <c r="X36" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2620,17 +2620,17 @@
       <c r="S37" s="2" t="n"/>
       <c r="T37" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U37" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U37" s="2" t="n"/>
       <c r="V37" s="2" t="n"/>
       <c r="W37" s="2" t="n"/>
-      <c r="X37" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X37" s="2" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2678,17 +2678,17 @@
       <c r="S38" s="2" t="n"/>
       <c r="T38" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U38" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U38" s="2" t="n"/>
       <c r="V38" s="2" t="n"/>
       <c r="W38" s="2" t="n"/>
-      <c r="X38" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X38" s="2" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2736,17 +2736,17 @@
       <c r="S39" s="2" t="n"/>
       <c r="T39" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U39" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U39" s="2" t="n"/>
       <c r="V39" s="2" t="n"/>
       <c r="W39" s="2" t="n"/>
-      <c r="X39" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2794,17 +2794,17 @@
       <c r="S40" s="2" t="n"/>
       <c r="T40" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U40" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U40" s="2" t="n"/>
       <c r="V40" s="2" t="n"/>
       <c r="W40" s="2" t="n"/>
-      <c r="X40" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X40" s="2" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2852,17 +2852,17 @@
       <c r="S41" s="2" t="n"/>
       <c r="T41" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U41" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U41" s="2" t="n"/>
       <c r="V41" s="2" t="n"/>
       <c r="W41" s="2" t="n"/>
-      <c r="X41" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X41" s="2" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2910,17 +2910,17 @@
       <c r="S42" s="2" t="n"/>
       <c r="T42" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U42" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U42" s="2" t="n"/>
       <c r="V42" s="2" t="n"/>
       <c r="W42" s="2" t="n"/>
-      <c r="X42" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X42" s="2" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2968,17 +2968,17 @@
       <c r="S43" s="2" t="n"/>
       <c r="T43" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U43" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U43" s="2" t="n"/>
       <c r="V43" s="2" t="n"/>
       <c r="W43" s="2" t="n"/>
-      <c r="X43" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X43" s="2" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3026,17 +3026,17 @@
       <c r="S44" s="2" t="n"/>
       <c r="T44" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U44" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U44" s="2" t="n"/>
       <c r="V44" s="2" t="n"/>
       <c r="W44" s="2" t="n"/>
-      <c r="X44" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3084,17 +3084,17 @@
       <c r="S45" s="2" t="n"/>
       <c r="T45" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U45" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U45" s="2" t="n"/>
       <c r="V45" s="2" t="n"/>
       <c r="W45" s="2" t="n"/>
-      <c r="X45" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X45" s="2" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3142,17 +3142,17 @@
       <c r="S46" s="2" t="n"/>
       <c r="T46" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U46" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U46" s="2" t="n"/>
       <c r="V46" s="2" t="n"/>
       <c r="W46" s="2" t="n"/>
-      <c r="X46" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X46" s="2" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3200,17 +3200,17 @@
       <c r="S47" s="2" t="n"/>
       <c r="T47" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U47" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U47" s="2" t="n"/>
       <c r="V47" s="2" t="n"/>
       <c r="W47" s="2" t="n"/>
-      <c r="X47" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X47" s="2" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3258,17 +3258,17 @@
       <c r="S48" s="2" t="n"/>
       <c r="T48" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U48" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U48" s="2" t="n"/>
       <c r="V48" s="2" t="n"/>
       <c r="W48" s="2" t="n"/>
-      <c r="X48" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X48" s="2" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3316,17 +3316,17 @@
       <c r="S49" s="2" t="n"/>
       <c r="T49" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U49" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U49" s="2" t="n"/>
       <c r="V49" s="2" t="n"/>
       <c r="W49" s="2" t="n"/>
-      <c r="X49" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X49" s="2" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3374,17 +3374,17 @@
       <c r="S50" s="2" t="n"/>
       <c r="T50" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U50" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U50" s="2" t="n"/>
       <c r="V50" s="2" t="n"/>
       <c r="W50" s="2" t="n"/>
-      <c r="X50" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X50" s="2" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3432,17 +3432,17 @@
       <c r="S51" s="2" t="n"/>
       <c r="T51" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U51" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U51" s="2" t="n"/>
       <c r="V51" s="2" t="n"/>
       <c r="W51" s="2" t="n"/>
-      <c r="X51" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X51" s="2" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3490,17 +3490,17 @@
       <c r="S52" s="2" t="n"/>
       <c r="T52" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U52" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U52" s="2" t="n"/>
       <c r="V52" s="2" t="n"/>
       <c r="W52" s="2" t="n"/>
-      <c r="X52" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X52" s="2" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3548,17 +3548,17 @@
       <c r="S53" s="2" t="n"/>
       <c r="T53" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U53" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U53" s="2" t="n"/>
       <c r="V53" s="2" t="n"/>
       <c r="W53" s="2" t="n"/>
-      <c r="X53" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X53" s="2" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3606,17 +3606,17 @@
       <c r="S54" s="2" t="n"/>
       <c r="T54" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U54" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U54" s="2" t="n"/>
       <c r="V54" s="2" t="n"/>
       <c r="W54" s="2" t="n"/>
-      <c r="X54" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X54" s="2" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3664,17 +3664,17 @@
       <c r="S55" s="2" t="n"/>
       <c r="T55" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U55" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U55" s="2" t="n"/>
       <c r="V55" s="2" t="n"/>
       <c r="W55" s="2" t="n"/>
-      <c r="X55" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X55" s="2" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3722,17 +3722,17 @@
       <c r="S56" s="2" t="n"/>
       <c r="T56" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U56" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U56" s="2" t="n"/>
       <c r="V56" s="2" t="n"/>
       <c r="W56" s="2" t="n"/>
-      <c r="X56" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X56" s="2" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3780,17 +3780,17 @@
       <c r="S57" s="2" t="n"/>
       <c r="T57" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U57" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U57" s="2" t="n"/>
       <c r="V57" s="2" t="n"/>
       <c r="W57" s="2" t="n"/>
-      <c r="X57" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X57" s="2" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3838,17 +3838,17 @@
       <c r="S58" s="2" t="n"/>
       <c r="T58" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U58" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U58" s="2" t="n"/>
       <c r="V58" s="2" t="n"/>
       <c r="W58" s="2" t="n"/>
-      <c r="X58" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X58" s="2" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -3896,17 +3896,17 @@
       <c r="S59" s="2" t="n"/>
       <c r="T59" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U59" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U59" s="2" t="n"/>
       <c r="V59" s="2" t="n"/>
       <c r="W59" s="2" t="n"/>
-      <c r="X59" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X59" s="2" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3972,21 +3972,21 @@
       </c>
       <c r="T60" s="2" t="inlineStr">
         <is>
+          <t>CM; JH; PS</t>
+        </is>
+      </c>
+      <c r="U60" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U60" s="2" t="inlineStr">
+      <c r="V60" s="2" t="n"/>
+      <c r="W60" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="V60" s="2" t="n"/>
-      <c r="W60" s="2" t="n"/>
-      <c r="X60" s="2" t="inlineStr">
-        <is>
-          <t>CM; JH; PS</t>
-        </is>
-      </c>
+      <c r="X60" s="2" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
@@ -4024,12 +4024,12 @@
       <c r="Q61" s="3" t="n"/>
       <c r="R61" s="3" t="n"/>
       <c r="S61" s="3" t="n"/>
-      <c r="T61" s="3" t="inlineStr">
+      <c r="T61" s="3" t="n"/>
+      <c r="U61" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U61" s="3" t="n"/>
       <c r="V61" s="3" t="n"/>
       <c r="W61" s="3" t="n"/>
       <c r="X61" s="3" t="n"/>
@@ -4070,12 +4070,12 @@
       <c r="Q62" s="3" t="n"/>
       <c r="R62" s="3" t="n"/>
       <c r="S62" s="3" t="n"/>
-      <c r="T62" s="3" t="inlineStr">
+      <c r="T62" s="3" t="n"/>
+      <c r="U62" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U62" s="3" t="n"/>
       <c r="V62" s="3" t="n"/>
       <c r="W62" s="3" t="n"/>
       <c r="X62" s="3" t="n"/>
@@ -4138,21 +4138,21 @@
       <c r="S63" s="2" t="n"/>
       <c r="T63" s="2" t="inlineStr">
         <is>
+          <t>CM; PS</t>
+        </is>
+      </c>
+      <c r="U63" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U63" s="2" t="inlineStr">
+      <c r="V63" s="2" t="n"/>
+      <c r="W63" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="V63" s="2" t="n"/>
-      <c r="W63" s="2" t="n"/>
-      <c r="X63" s="2" t="inlineStr">
-        <is>
-          <t>CM; PS</t>
-        </is>
-      </c>
+      <c r="X63" s="2" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
@@ -4192,21 +4192,21 @@
       <c r="S64" s="3" t="n"/>
       <c r="T64" s="3" t="inlineStr">
         <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="U64" s="3" t="inlineStr">
+        <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U64" s="3" t="inlineStr">
+      <c r="V64" s="3" t="n"/>
+      <c r="W64" s="3" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="V64" s="3" t="n"/>
-      <c r="W64" s="3" t="n"/>
-      <c r="X64" s="3" t="inlineStr">
-        <is>
-          <t>CM</t>
-        </is>
-      </c>
+      <c r="X64" s="3" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
@@ -4246,21 +4246,21 @@
       <c r="S65" s="3" t="n"/>
       <c r="T65" s="3" t="inlineStr">
         <is>
+          <t>CM; RW</t>
+        </is>
+      </c>
+      <c r="U65" s="3" t="inlineStr">
+        <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U65" s="3" t="inlineStr">
+      <c r="V65" s="3" t="n"/>
+      <c r="W65" s="3" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="V65" s="3" t="n"/>
-      <c r="W65" s="3" t="n"/>
-      <c r="X65" s="3" t="inlineStr">
-        <is>
-          <t>CM; RW</t>
-        </is>
-      </c>
+      <c r="X65" s="3" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -4317,21 +4317,21 @@
       <c r="S66" s="2" t="n"/>
       <c r="T66" s="2" t="inlineStr">
         <is>
+          <t>CM; JH; PS</t>
+        </is>
+      </c>
+      <c r="U66" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U66" s="2" t="inlineStr">
+      <c r="V66" s="2" t="n"/>
+      <c r="W66" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="V66" s="2" t="n"/>
-      <c r="W66" s="2" t="n"/>
-      <c r="X66" s="2" t="inlineStr">
-        <is>
-          <t>CM; JH; PS</t>
-        </is>
-      </c>
+      <c r="X66" s="2" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
@@ -4382,12 +4382,12 @@
       <c r="Q67" s="3" t="n"/>
       <c r="R67" s="3" t="n"/>
       <c r="S67" s="3" t="n"/>
-      <c r="T67" s="3" t="inlineStr">
+      <c r="T67" s="3" t="n"/>
+      <c r="U67" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U67" s="3" t="n"/>
       <c r="V67" s="3" t="n"/>
       <c r="W67" s="3" t="n"/>
       <c r="X67" s="3" t="n"/>
@@ -4430,21 +4430,21 @@
       <c r="S68" s="3" t="n"/>
       <c r="T68" s="3" t="inlineStr">
         <is>
+          <t>CM; RW</t>
+        </is>
+      </c>
+      <c r="U68" s="3" t="inlineStr">
+        <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U68" s="3" t="inlineStr">
+      <c r="V68" s="3" t="n"/>
+      <c r="W68" s="3" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="V68" s="3" t="n"/>
-      <c r="W68" s="3" t="n"/>
-      <c r="X68" s="3" t="inlineStr">
-        <is>
-          <t>CM; RW</t>
-        </is>
-      </c>
+      <c r="X68" s="3" t="n"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4469,12 +4469,12 @@
       </c>
       <c r="T69" t="inlineStr">
         <is>
+          <t>JH; PS</t>
+        </is>
+      </c>
+      <c r="U69" t="inlineStr">
+        <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="X69" t="inlineStr">
-        <is>
-          <t>JH; PS</t>
         </is>
       </c>
     </row>
@@ -4517,17 +4517,17 @@
       <c r="S70" s="3" t="n"/>
       <c r="T70" s="3" t="inlineStr">
         <is>
+          <t>JH</t>
+        </is>
+      </c>
+      <c r="U70" s="3" t="inlineStr">
+        <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U70" s="3" t="n"/>
       <c r="V70" s="3" t="n"/>
       <c r="W70" s="3" t="n"/>
-      <c r="X70" s="3" t="inlineStr">
-        <is>
-          <t>JH</t>
-        </is>
-      </c>
+      <c r="X70" s="3" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
@@ -4571,17 +4571,17 @@
       <c r="S71" s="3" t="n"/>
       <c r="T71" s="3" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U71" s="3" t="inlineStr">
+        <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U71" s="3" t="n"/>
       <c r="V71" s="3" t="n"/>
       <c r="W71" s="3" t="n"/>
-      <c r="X71" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="X71" s="3" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4644,21 +4644,21 @@
       <c r="S72" s="2" t="n"/>
       <c r="T72" s="2" t="inlineStr">
         <is>
+          <t>CM; JH; PS</t>
+        </is>
+      </c>
+      <c r="U72" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U72" s="2" t="inlineStr">
+      <c r="V72" s="2" t="n"/>
+      <c r="W72" s="2" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="V72" s="2" t="n"/>
-      <c r="W72" s="2" t="n"/>
-      <c r="X72" s="2" t="inlineStr">
-        <is>
-          <t>CM; JH; PS</t>
-        </is>
-      </c>
+      <c r="X72" s="2" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
@@ -4714,12 +4714,12 @@
       <c r="Q73" s="3" t="n"/>
       <c r="R73" s="3" t="n"/>
       <c r="S73" s="3" t="n"/>
-      <c r="T73" s="3" t="inlineStr">
+      <c r="T73" s="3" t="n"/>
+      <c r="U73" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U73" s="3" t="n"/>
       <c r="V73" s="3" t="n"/>
       <c r="W73" s="3" t="n"/>
       <c r="X73" s="3" t="n"/>
@@ -4755,7 +4755,7 @@
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
         </is>
       </c>
-      <c r="G74" s="3" t="inlineStr"/>
+      <c r="G74" s="3" t="n"/>
       <c r="H74" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Use this entity when authors describe the total amount of contact time for a particular part/intervention across multiple contact events. 
@@ -4793,23 +4793,23 @@
       </c>
       <c r="T74" s="3" t="inlineStr">
         <is>
+          <t>CM; JH; PS</t>
+        </is>
+      </c>
+      <c r="U74" s="3" t="inlineStr">
+        <is>
           <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="U74" s="3" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="V74" s="3" t="n"/>
       <c r="W74" s="3" t="inlineStr">
         <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="X74" s="3" t="inlineStr">
+        <is>
           <t>what type of data item is this? (CM)</t>
-        </is>
-      </c>
-      <c r="X74" s="3" t="inlineStr">
-        <is>
-          <t>CM; JH; PS</t>
         </is>
       </c>
     </row>
@@ -4849,12 +4849,12 @@
       <c r="Q75" s="3" t="n"/>
       <c r="R75" s="3" t="n"/>
       <c r="S75" s="3" t="n"/>
-      <c r="T75" s="3" t="inlineStr">
+      <c r="T75" s="3" t="n"/>
+      <c r="U75" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U75" s="3" t="n"/>
       <c r="V75" s="3" t="n"/>
       <c r="W75" s="3" t="n"/>
       <c r="X75" s="3" t="n"/>
@@ -4880,7 +4880,11 @@
           <t>data item</t>
         </is>
       </c>
-      <c r="E76" s="2" t="n"/>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The planned total duration of all sessions or digital contacts in an intervention or part. </t>
+        </is>
+      </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
           <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
@@ -4907,7 +4911,7 @@
           <t>intervention contact event</t>
         </is>
       </c>
-      <c r="M76" s="2" t="inlineStr"/>
+      <c r="M76" s="2" t="n"/>
       <c r="N76" s="2" t="n"/>
       <c r="O76" s="2" t="n"/>
       <c r="P76" s="2" t="n"/>
@@ -4916,17 +4920,17 @@
       <c r="S76" s="2" t="n"/>
       <c r="T76" s="2" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U76" s="2" t="inlineStr">
+        <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="U76" s="2" t="n"/>
-      <c r="V76" s="2" t="inlineStr"/>
-      <c r="W76" s="2" t="inlineStr"/>
-      <c r="X76" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="V76" s="2" t="n"/>
+      <c r="W76" s="2" t="n"/>
+      <c r="X76" s="2" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
@@ -4978,23 +4982,23 @@
       </c>
       <c r="T77" s="3" t="inlineStr">
         <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="U77" s="3" t="inlineStr">
+        <is>
           <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="U77" s="3" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="V77" s="3" t="n"/>
       <c r="W77" s="3" t="inlineStr">
         <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="X77" s="3" t="inlineStr">
+        <is>
           <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described (CM)</t>
-        </is>
-      </c>
-      <c r="X77" s="3" t="inlineStr">
-        <is>
-          <t>CM</t>
         </is>
       </c>
     </row>
@@ -5056,23 +5060,23 @@
       </c>
       <c r="T78" s="3" t="inlineStr">
         <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="U78" s="3" t="inlineStr">
+        <is>
           <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="U78" s="3" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="V78" s="3" t="n"/>
       <c r="W78" s="3" t="inlineStr">
         <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="X78" s="3" t="inlineStr">
+        <is>
           <t>meeting was cut short whilst JH gave feedback on these entities. JH, please could you give feedback here? I think the suggestion was to combine these two entities (BCIO:008550 and BCIO:008555)</t>
-        </is>
-      </c>
-      <c r="X78" s="3" t="inlineStr">
-        <is>
-          <t>CM</t>
         </is>
       </c>
     </row>
@@ -5134,23 +5138,23 @@
       </c>
       <c r="T79" s="3" t="inlineStr">
         <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="U79" s="3" t="inlineStr">
+        <is>
           <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="U79" s="3" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="V79" s="3" t="n"/>
       <c r="W79" s="3" t="inlineStr">
         <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="X79" s="3" t="inlineStr">
+        <is>
           <t>meeting was cut short whilst JH gave feedback on these entities. JH, please could you give feedback here? I think the suggestion was to combine these two entities (BCIO:008550 and BCIO:008555)</t>
-        </is>
-      </c>
-      <c r="X79" s="3" t="inlineStr">
-        <is>
-          <t>CM</t>
         </is>
       </c>
     </row>
@@ -5204,23 +5208,23 @@
       </c>
       <c r="T80" s="3" t="inlineStr">
         <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="U80" s="3" t="inlineStr">
+        <is>
           <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="U80" s="3" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="V80" s="3" t="n"/>
       <c r="W80" s="3" t="inlineStr">
         <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="X80" s="3" t="inlineStr">
+        <is>
           <t>this entity was added to allow us to more flexibly capture frequencies that have been broken down into period and repetitions. This is useful for annotations but we are unsure if it makes ontological sense to include it as it isn't really distinct from a frequency itself and relates more to how a frequency is described. Perhaps this also isn't really distinct from duration of BCI/part (CM)</t>
-        </is>
-      </c>
-      <c r="X80" s="3" t="inlineStr">
-        <is>
-          <t>CM</t>
         </is>
       </c>
     </row>
@@ -5262,21 +5266,21 @@
       <c r="S81" s="3" t="n"/>
       <c r="T81" s="3" t="inlineStr">
         <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="U81" s="3" t="inlineStr">
+        <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="U81" s="3" t="inlineStr">
+      <c r="V81" s="3" t="n"/>
+      <c r="W81" s="3" t="inlineStr">
         <is>
           <t>JH, SM, RW</t>
         </is>
       </c>
-      <c r="V81" s="3" t="n"/>
-      <c r="W81" s="3" t="n"/>
-      <c r="X81" s="3" t="inlineStr">
-        <is>
-          <t>CM</t>
-        </is>
-      </c>
+      <c r="X81" s="3" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
@@ -5334,23 +5338,23 @@
       </c>
       <c r="T82" s="3" t="inlineStr">
         <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="U82" s="3" t="inlineStr">
+        <is>
           <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="U82" s="3" t="inlineStr">
-        <is>
-          <t>JH, SM, RW</t>
         </is>
       </c>
       <c r="V82" s="3" t="n"/>
       <c r="W82" s="3" t="inlineStr">
         <is>
+          <t>JH, SM, RW</t>
+        </is>
+      </c>
+      <c r="X82" s="3" t="inlineStr">
+        <is>
           <t>need to decide whether to have a separate additional entity for frequency of contact events (CM)</t>
-        </is>
-      </c>
-      <c r="X82" s="3" t="inlineStr">
-        <is>
-          <t>CM</t>
         </is>
       </c>
     </row>

</xml_diff>